<commit_message>
Previsibilidade de receita: pipeline ponderado e run-rate do CRM (aba Previsao_Receita, página 4 do painel e slide 3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/omie-case-contadores/output/Desafio3_Capacity.xlsx
+++ b/omie-case-contadores/output/Desafio3_Capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f75accf49a20a1b0/Documentos/Omie_Antigravity/omie-case-contadores/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_455B2EBFF673AF22A527CC428010DD7A4F814E1A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_455B6DB736781122A527CC428010DD7A4F814E1A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2299,7 +2299,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-A576-4246-93BD-C8EBB6E5A38C}"/>
+              <c16:uniqueId val="{00000000-0E6F-416C-8173-17F185491A08}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
Avaliação do D2 em 3 perguntas (target, real, piloto) no Excel e no painel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/omie-case-contadores/output/Desafio3_Capacity.xlsx
+++ b/omie-case-contadores/output/Desafio3_Capacity.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f75accf49a20a1b0/Documentos/Omie_Antigravity/omie-case-contadores/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_38E3365F1244E93363025DC9B21CC5521A8C1452" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_38E3A6D75377A13363025DC9B21CC5521A8C1452" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2329,7 +2329,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5A14-41FB-BAF0-C80006CBE9F5}"/>
+              <c16:uniqueId val="{00000000-4775-498B-8ECE-7E6794029E93}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>